<commit_message>
chore: sync live Excel and CSV exports
</commit_message>
<xml_diff>
--- a/TMS_Completed_Claims.xlsx
+++ b/TMS_Completed_Claims.xlsx
@@ -1811,12 +1811,12 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1826,17 +1826,17 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>21:32:20</t>
+          <t>16:30:32</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>22:18:08</t>
+          <t>17:29:09</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>00:45:48</t>
+          <t>00:58:37</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -1888,12 +1888,12 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1903,17 +1903,17 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>22:18:08</t>
+          <t>17:29:09</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>22:54:46</t>
+          <t>18:16:03</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>00:36:38</t>
+          <t>00:46:54</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -1965,12 +1965,12 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1980,17 +1980,17 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>22:54:46</t>
+          <t>18:16:03</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>00:08:03</t>
+          <t>19:49:51</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>01:13:17</t>
+          <t>01:33:48</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2042,12 +2042,12 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -2057,17 +2057,17 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>00:08:03</t>
+          <t>19:49:51</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>01:57:59</t>
+          <t>22:10:33</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>01:49:56</t>
+          <t>02:20:42</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2119,12 +2119,12 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -2134,17 +2134,17 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>01:57:59</t>
+          <t>22:10:33</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>03:29:36</t>
+          <t>00:07:48</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>01:31:37</t>
+          <t>01:57:15</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2196,12 +2196,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2211,17 +2211,17 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>03:29:36</t>
+          <t>00:07:48</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>04:15:24</t>
+          <t>01:06:25</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>00:45:48</t>
+          <t>00:58:37</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2273,12 +2273,12 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -2288,17 +2288,17 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>04:15:24</t>
+          <t>01:06:25</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>04:52:02</t>
+          <t>01:53:19</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>00:36:38</t>
+          <t>00:46:54</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2350,12 +2350,12 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -2365,17 +2365,17 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>04:52:02</t>
+          <t>01:53:19</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>05:56:10</t>
+          <t>03:15:23</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>01:04:08</t>
+          <t>01:22:04</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2427,12 +2427,12 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>05:56:10</t>
+          <t>03:15:23</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>07:09:27</t>
+          <t>04:49:11</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>01:13:17</t>
+          <t>01:33:48</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2504,12 +2504,12 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>07:09:27</t>
+          <t>04:49:11</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>08:22:44</t>
+          <t>06:22:59</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>01:13:17</t>
+          <t>01:33:48</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2581,12 +2581,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -2596,17 +2596,17 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>08:22:44</t>
+          <t>06:22:59</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>10:31:00</t>
+          <t>09:07:08</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>02:08:16</t>
+          <t>02:44:09</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2658,12 +2658,12 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -2673,17 +2673,17 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>10:31:00</t>
+          <t>09:07:08</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>12:20:56</t>
+          <t>11:27:50</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>01:49:56</t>
+          <t>02:20:42</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2735,12 +2735,12 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -2750,17 +2750,17 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>12:20:56</t>
+          <t>11:27:50</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>13:15:54</t>
+          <t>12:38:11</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>00:54:58</t>
+          <t>01:10:21</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2812,12 +2812,12 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -2827,17 +2827,17 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>13:15:54</t>
+          <t>12:38:11</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>14:29:11</t>
+          <t>14:11:59</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>01:13:17</t>
+          <t>01:33:48</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2889,12 +2889,12 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -2904,17 +2904,17 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>14:29:11</t>
+          <t>14:11:59</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>15:05:49</t>
+          <t>14:58:53</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>00:36:38</t>
+          <t>00:46:54</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="O32" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -2966,12 +2966,12 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>GWH-Cigna</t>
+          <t>UHC</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>CLM-003</t>
+          <t>CLM-002</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -2981,17 +2981,17 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>15:05:49</t>
+          <t>14:58:53</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>15:33:18</t>
+          <t>15:34:03</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>00:27:29</t>
+          <t>00:35:10</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>sess-a27a8025</t>
+          <t>sess-851ec4f9</t>
         </is>
       </c>
     </row>
@@ -3043,12 +3043,12 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -3058,17 +3058,17 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>16:30:32</t>
+          <t>21:32:20</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>17:29:09</t>
+          <t>22:21:55</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>00:58:37</t>
+          <t>00:49:35</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3120,12 +3120,12 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -3135,17 +3135,17 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>17:29:09</t>
+          <t>22:21:55</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>18:16:03</t>
+          <t>23:01:35</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>00:46:54</t>
+          <t>00:39:40</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3197,12 +3197,12 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -3212,17 +3212,17 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>18:16:03</t>
+          <t>23:01:35</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>19:49:51</t>
+          <t>00:20:55</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>01:33:48</t>
+          <t>01:19:20</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3274,12 +3274,12 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -3289,17 +3289,17 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>19:49:51</t>
+          <t>00:20:55</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>22:10:33</t>
+          <t>02:19:55</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>02:20:42</t>
+          <t>01:59:00</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="O37" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3351,12 +3351,12 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -3366,17 +3366,17 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>22:10:33</t>
+          <t>02:19:55</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>00:07:48</t>
+          <t>03:59:05</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>01:57:15</t>
+          <t>01:39:10</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="O38" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3428,12 +3428,12 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -3443,17 +3443,17 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>00:07:48</t>
+          <t>03:59:05</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>01:06:25</t>
+          <t>04:48:40</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>00:58:37</t>
+          <t>00:49:35</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="O39" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3505,12 +3505,12 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -3520,17 +3520,17 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>01:06:25</t>
+          <t>04:48:40</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>01:53:19</t>
+          <t>05:28:20</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>00:46:54</t>
+          <t>00:39:40</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="O40" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3582,12 +3582,12 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -3597,17 +3597,17 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>01:53:19</t>
+          <t>05:28:20</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>03:15:23</t>
+          <t>06:37:45</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>01:22:04</t>
+          <t>01:09:25</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="O41" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3659,12 +3659,12 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -3674,17 +3674,17 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>03:15:23</t>
+          <t>06:37:45</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>04:49:11</t>
+          <t>07:57:05</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>01:33:48</t>
+          <t>01:19:20</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="O42" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3736,12 +3736,12 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -3751,17 +3751,17 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>04:49:11</t>
+          <t>07:57:05</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>06:22:59</t>
+          <t>09:16:25</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>01:33:48</t>
+          <t>01:19:20</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="O43" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3813,12 +3813,12 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -3828,17 +3828,17 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>06:22:59</t>
+          <t>09:16:25</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>09:07:08</t>
+          <t>11:35:16</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>02:44:09</t>
+          <t>02:18:51</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="O44" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3890,12 +3890,12 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -3905,17 +3905,17 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>09:07:08</t>
+          <t>11:35:16</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>11:27:50</t>
+          <t>13:34:16</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>02:20:42</t>
+          <t>01:59:00</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -3967,12 +3967,12 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -3982,17 +3982,17 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>11:27:50</t>
+          <t>13:34:16</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>12:38:11</t>
+          <t>14:33:46</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>01:10:21</t>
+          <t>00:59:30</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4022,7 +4022,7 @@
       </c>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -4044,12 +4044,12 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -4059,17 +4059,17 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>12:38:11</t>
+          <t>14:33:46</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>14:11:59</t>
+          <t>15:53:06</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>01:33:48</t>
+          <t>01:19:20</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="O47" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -4121,12 +4121,12 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -4136,17 +4136,17 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>14:11:59</t>
+          <t>15:53:06</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>14:58:53</t>
+          <t>16:32:46</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>00:46:54</t>
+          <t>00:39:40</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="O48" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>
@@ -4198,12 +4198,12 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>UHC</t>
+          <t>GWH-Cigna</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>CLM-002</t>
+          <t>CLM-003</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -4213,17 +4213,17 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>14:58:53</t>
+          <t>16:32:46</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>15:34:03</t>
+          <t>17:02:31</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>00:35:10</t>
+          <t>00:29:45</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="O49" s="3" t="inlineStr">
         <is>
-          <t>sess-851ec4f9</t>
+          <t>sess-a27a8025</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: save updated completed claims excel and csv
</commit_message>
<xml_diff>
--- a/TMS_Completed_Claims.xlsx
+++ b/TMS_Completed_Claims.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4257,6 +4257,1315 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Login to Citrix application.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>21:11:59</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>21:13:20</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>00:01:21</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O50" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Login to Athena software.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>21:13:20</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>21:14:25</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>00:01:05</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O51" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Search and open the assigned Claim ID in Athena.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>21:14:25</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>21:16:35</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>00:02:10</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O52" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Review claim details, denial reason, notes history, and billing information.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>21:16:35</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>21:19:50</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>00:03:15</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O53" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Perform pre-service/claim analysis to identify the next action.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>21:19:50</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>21:22:32</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>00:02:42</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O54" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Open the Phone Payer tab in Athena.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>21:22:32</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>21:23:53</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>00:01:21</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O55" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Verify payer information and available contact details.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>21:23:53</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>21:24:58</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>00:01:05</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O56" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Review policy guidelines; pause for supervisor override authorization.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>21:24:58</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>21:28:13</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>00:03:15</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>NVA</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O57" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Login to portal.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>21:28:13</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>21:30:06</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>00:01:53</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O58" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Cross-reference patient eligibility across clearinghouse portals.</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>21:30:06</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>21:32:16</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>00:02:10</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>NVA</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O59" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Review any available EOB, Previous, or documents.</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>21:32:16</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>21:34:26</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>00:02:10</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O60" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>A call is placed to the Insurance</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>21:34:26</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>21:38:13</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>00:03:47</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O61" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Discuss about the claim/appeal/Reprocess status with the insurance representative</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>21:38:13</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>21:41:28</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>00:03:15</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O62" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Take the information from the representative</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>21:41:28</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>21:43:05</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>00:01:37</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O63" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Update detailed call notes in Athena.</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>21:43:05</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>21:45:15</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>00:02:10</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O64" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Validate that all supporting information has been documented accurately.</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>21:45:15</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>21:46:20</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>00:01:05</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O65" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>CLM-007</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>Save all changes and move to the next claim.</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>21:46:20</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>21:47:08</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>00:00:48</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O66" s="3" t="inlineStr">
+        <is>
+          <t>sess-734d32a9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed: dialog box bugs and errors
</commit_message>
<xml_diff>
--- a/TMS_Completed_Claims.xlsx
+++ b/TMS_Completed_Claims.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O66"/>
+  <dimension ref="A1:O81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5566,6 +5566,1161 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Login to Citrix application.</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>15:34:18</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>02:25:48</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>10:51:30</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O67" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Login to Athena software.</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>02:25:48</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>11:07:00</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>08:41:12</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O68" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>Search and open the assigned Claim ID in Athena.</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>11:07:00</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>04:29:25</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>17:22:25</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O69" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Review claim details, denial reason, notes history, and billing information.</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>04:29:25</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>06:33:03</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>26:03:38</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O70" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Perform pre-service/claim analysis to identify the next action.</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>06:33:03</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>04:16:04</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>21:43:01</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O71" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Open the Phone Payer tab in Athena.</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>04:16:04</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>15:07:34</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>10:51:30</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O72" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Verify payer information and available contact details.</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>15:07:34</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>23:48:46</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>08:41:12</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O73" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>Login to portal.</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>23:48:46</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>15:00:53</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>15:12:07</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O74" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>Review any available EOB, Previous, or documents.</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>15:00:53</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>08:23:18</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>17:22:25</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O75" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>A call is placed to the Insurance</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>08:23:18</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>14:47:32</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>30:24:14</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O76" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>Discuss about the claim/appeal/Reprocess status with the insurance representative</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>14:47:32</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>16:51:10</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>26:03:38</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O77" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>Take the information from the representative</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>16:51:10</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>05:52:59</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>13:01:49</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O78" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Update detailed call notes in Athena.</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>05:52:59</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>23:15:24</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>17:22:25</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O79" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Validate that all supporting information has been documented accurately.</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>23:15:24</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>07:56:36</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>08:41:12</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O80" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>CLM-005</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Save all changes and move to the next claim.</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>07:56:36</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>14:27:30</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>06:30:54</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O81" s="3" t="inlineStr">
+        <is>
+          <t>sess-ed07904f</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed: AHT and dialog box
</commit_message>
<xml_diff>
--- a/TMS_Completed_Claims.xlsx
+++ b/TMS_Completed_Claims.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O81"/>
+  <dimension ref="A1:O97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6721,6 +6721,1238 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Login to Citrix application.</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>11:03:35</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>11:03:50</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>00:00:15</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O82" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Login to Athena software.</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>11:03:50</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>11:04:02</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>00:00:12</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O83" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>Search and open the assigned Claim ID in Athena.</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>11:04:02</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>11:04:27</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>00:00:25</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O84" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Review claim details, denial reason, notes history, and billing information.</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>11:04:27</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>11:05:05</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>00:00:38</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O85" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>Perform pre-service/claim analysis to identify the next action.</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>11:05:05</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>11:05:36</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>00:00:31</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O86" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>Open the Phone Payer tab in Athena.</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>11:05:36</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>11:05:51</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>00:00:15</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O87" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>Verify payer information and available contact details.</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>11:05:51</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>11:06:03</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>00:00:12</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O88" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>Login to portal.</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>11:06:03</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>11:06:25</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>00:00:22</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O89" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>Cross-reference patient eligibility across clearinghouse portals.</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>11:06:25</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>11:06:50</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>00:00:25</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>NVA</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O90" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>Review any available EOB, Previous, or documents.</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>11:06:50</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>11:07:15</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>00:00:25</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O91" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>A call is placed to the Insurance</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>11:07:15</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>11:07:59</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>00:00:44</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O92" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>Discuss about the claim/appeal/Reprocess status with the insurance representative</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>11:07:59</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>11:08:37</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>00:00:38</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O93" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>Take the information from the representative</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>11:08:37</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>11:08:56</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>00:00:19</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O94" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>Update detailed call notes in Athena.</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>11:08:56</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>11:09:21</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>00:00:25</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O95" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>Validate that all supporting information has been documented accurately.</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>11:09:21</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>11:09:33</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>00:00:12</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O96" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>CLM-2233</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>Save all changes and move to the next claim.</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>11:09:33</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>11:09:42</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>00:00:09</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O97" s="3" t="inlineStr">
+        <is>
+          <t>sess-5d3be309</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(telemetry): complete end-to-end dialog triggering, strict claim validation, live AHT tracking, and Excel sync
</commit_message>
<xml_diff>
--- a/TMS_Completed_Claims.xlsx
+++ b/TMS_Completed_Claims.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O97"/>
+  <dimension ref="A1:O112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7953,6 +7953,1161 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>Login to Citrix application.</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>21:06:56</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>21:07:09</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>00:00:13</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O98" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>Login to Athena software.</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>21:07:09</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>21:07:19</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>00:00:10</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O99" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>Search and open the assigned Claim ID in Athena.</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>21:07:19</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>21:07:40</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>00:00:21</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O100" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>Review claim details, denial reason, notes history, and billing information.</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>21:07:40</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>21:08:12</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>00:00:32</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O101" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>Perform pre-service/claim analysis to identify the next action.</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>21:08:12</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>21:08:39</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>00:00:27</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O102" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t>Open the Phone Payer tab in Athena.</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>21:08:39</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>21:08:52</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>00:00:13</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O103" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>Verify payer information and available contact details.</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>21:08:52</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>21:09:02</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>00:00:10</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O104" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>Login to portal.</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>21:09:02</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>21:09:21</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>00:00:19</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N105" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O105" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>Review any available EOB, Previous, or documents.</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>21:09:21</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>21:09:42</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>00:00:21</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O106" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>A call is placed to the Insurance</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>21:09:42</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>21:10:20</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>00:00:38</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O107" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>Discuss about the claim/appeal/Reprocess status with the insurance representative</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>21:10:20</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>21:10:52</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>00:00:32</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O108" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>Take the information from the representative</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>21:10:52</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>21:11:08</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>00:00:16</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O109" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>Update detailed call notes in Athena.</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>21:11:08</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>21:11:29</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>00:00:21</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O110" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>Validate that all supporting information has been documented accurately.</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>21:11:29</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>21:11:39</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>00:00:10</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N111" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O111" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Associate EMP101</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>Prev Entd</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>UHC</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>CLM-605</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>Save all changes and move to the next claim.</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>21:11:39</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>21:11:47</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>00:00:08</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
+          <t>Tenured</t>
+        </is>
+      </c>
+      <c r="O112" s="3" t="inlineStr">
+        <is>
+          <t>sess-emp101-1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>